<commit_message>
feat(rh): KB treinamentos com capturas reais, dark mode e diagnosticos locais
Adiciona base de conhecimento operacional (/rh/treinamentos) com 9 artigos e PNGs reais, tema claro/escuro no layout, scripts de diagnostico/import de contrato e enrichment MTR ao abrir faturamento — sem alterar logica congelada.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/relatorios/contrato-fila-faturamento-2026-06-11.xlsx
+++ b/docs/relatorios/contrato-fila-faturamento-2026-06-11.xlsx
@@ -5120,22 +5120,22 @@
         <v/>
       </c>
       <c r="K63" t="str">
-        <v>VALOR_ZERO_NO_CONTRATO</v>
+        <v>SEM_MATCH_RESIDUO</v>
       </c>
       <c r="L63" t="str">
-        <v>TROCA CAÇAMBA 7M³ - LODO</v>
-      </c>
-      <c r="M63">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="M63" t="str">
+        <v/>
       </c>
       <c r="N63" t="str">
         <v/>
       </c>
       <c r="O63" t="str">
-        <v>kg</v>
+        <v/>
       </c>
       <c r="P63" t="str">
-        <v>TROCA CAÇAMBA 7M³ - LODO (R$ 0/un)</v>
+        <v>LODO DE ESTAÇÃO DE TRATAMENTO (R$ 0/un)</v>
       </c>
       <c r="Q63" t="str">
         <v/>
@@ -5144,7 +5144,7 @@
         <v>aguardando aprovação do Faturamento, sem valor</v>
       </c>
       <c r="S63" t="str">
-        <v>Preencher valor (R$/kg ou unidade) no cadastro do cliente e salvar</v>
+        <v>Conferir nome do resíduo na coleta vs cadastro do cliente</v>
       </c>
       <c r="T63" t="str">
         <v>TROCA CAÇAMBA 7M³ - LODO</v>
@@ -15943,16 +15943,16 @@
         <v>1</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
       <c r="G28" t="str">
-        <v>TROCA CAÇAMBA 7M³ - LODO (R$ 0/un)</v>
+        <v>LODO DE ESTAÇÃO DE TRATAMENTO (R$ 0/un)</v>
       </c>
     </row>
     <row r="29">

</xml_diff>